<commit_message>
update 17 agosto corretta
</commit_message>
<xml_diff>
--- a/Survey_data_real.xlsx
+++ b/Survey_data_real.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Other computers\My Laptop (1)\Other\ShinyAPPnorway\ACCESS-FjordAPP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{734DDD04-CCB8-47BC-B11D-362EF8DBCC84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55B8E29A-375B-47D9-AFB9-1A8952A2FA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18,7 +18,7 @@
     <sheet name="stratum_info" sheetId="2" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">catchdata!$A$1:$J$118</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">catchdata!$A$1:$J$180</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">station_info!$A$1:$S$216</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -4689,7 +4689,7 @@
         <v>54</v>
       </c>
       <c r="C165" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D165" t="s">
         <v>96</v>

</xml_diff>